<commit_message>
Stream long-form model points through value_file
value_file now mirrors read_model_points -- with the new `coverages`
argument it streams a long-form policies + coverages pair, chunking the
policies and pulling each chunk's coverage rows by `policy_id`, not just
a wide parquet.

Reorder the riders sheet to `product, rider_code, rider_name, type` and
regenerate the bundled sample.
</commit_message>
<xml_diff>
--- a/src/fastcashflow/sample_data/sample_assumptions.xlsx
+++ b/src/fastcashflow/sample_data/sample_assumptions.xlsx
@@ -2316,17 +2316,17 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>product</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>rider_code</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>rider_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>product</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -2338,17 +2338,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>DTH_MAIN</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>주계약사망</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>-</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -2360,17 +2360,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ADB</t>
+          <t>-</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>ADB</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>재해사망특약</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>-</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -2382,17 +2382,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HOSP</t>
+          <t>-</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>HOSP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>입원특약</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>-</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -2404,17 +2404,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CANCER</t>
+          <t>-</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>CANCER</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>암진단특약</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>-</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -2426,17 +2426,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>ANN</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>연금특약</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>-</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2448,17 +2448,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>MAT</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>생존특약</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>-</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">

</xml_diff>

<commit_message>
rename product code convention to SCREAMING_SNAKE_CASE (term_a -> TERM_A)
Align 'product' with the table_id / channel uppercase family so the
sample workbook and every doc / test stops mixing lowercase product
with uppercase everything else. naming-conventions.md and
design-decisions.md flipped to the new rule; bundled sample workbook
and policies CSV updated alongside.
</commit_message>
<xml_diff>
--- a/src/fastcashflow/sample_data/sample_assumptions.xlsx
+++ b/src/fastcashflow/sample_data/sample_assumptions.xlsx
@@ -540,7 +540,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>term_a</t>
+          <t>TERM_A</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -560,7 +560,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>term_a</t>
+          <t>TERM_A</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -621,7 +621,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>term_a</t>
+          <t>TERM_A</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -643,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>term_a</t>
+          <t>TERM_A</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -670,7 +670,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>term_a</t>
+          <t>TERM_A</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -697,7 +697,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>term_a</t>
+          <t>TERM_A</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -724,7 +724,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>term_a</t>
+          <t>TERM_A</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -746,7 +746,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>term_a</t>
+          <t>TERM_A</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">

</xml_diff>

<commit_message>
refactor!: rename expense basis to alpha/beta/gamma + LAE convention
Adopt Korean actuarial alpha / beta / gamma naming for ExpenseRow.basis
plus a dedicated LAE (Loss Adjustment Expense) slot:

  premium_pct_init    -> alpha_pro_rata
  per_policy_init     -> alpha_fixed
  premium_pct         -> beta_pro_rata
  per_policy_monthly  -> gamma_fixed
  claim_pct           -> lae_pro_rata

The pro_rata / fixed suffixes make the dispatch meaning explicit -- the
old *_pct names suggested percent but stored fractions, and were silent
on the base. lae_pro_rata names the slot after the LAE standard term
rather than the bag-word "claim handling".

Kernel-internal variables, codegen strings, sample workbook
expense_tables sheet, all test fixtures and docs migrate together.
390 tests pass.
</commit_message>
<xml_diff>
--- a/src/fastcashflow/sample_data/sample_assumptions.xlsx
+++ b/src/fastcashflow/sample_data/sample_assumptions.xlsx
@@ -499,7 +499,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>per_policy_init</t>
+          <t>alpha_fixed</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -519,7 +519,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>per_policy_monthly</t>
+          <t>gamma_fixed</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -539,7 +539,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>per_policy_init</t>
+          <t>alpha_fixed</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -559,7 +559,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>per_policy_monthly</t>
+          <t>gamma_fixed</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -579,7 +579,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>per_policy_init</t>
+          <t>alpha_fixed</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -599,7 +599,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>per_policy_monthly</t>
+          <t>gamma_fixed</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -619,7 +619,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>per_policy_init</t>
+          <t>alpha_fixed</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -639,7 +639,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>per_policy_monthly</t>
+          <t>gamma_fixed</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -659,7 +659,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>per_policy_init</t>
+          <t>alpha_fixed</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -679,7 +679,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>per_policy_monthly</t>
+          <t>gamma_fixed</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -699,7 +699,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>per_policy_init</t>
+          <t>alpha_fixed</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -719,7 +719,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>per_policy_monthly</t>
+          <t>gamma_fixed</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -739,7 +739,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>per_policy_init</t>
+          <t>alpha_fixed</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -759,7 +759,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>per_policy_monthly</t>
+          <t>gamma_fixed</t>
         </is>
       </c>
       <c r="D15" t="n">

</xml_diff>